<commit_message>
commit logic submit product
</commit_message>
<xml_diff>
--- a/draw-design/code_nam_value.xlsx
+++ b/draw-design/code_nam_value.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="49">
   <si>
     <t>CodeCd</t>
   </si>
@@ -89,6 +89,78 @@
   </si>
   <si>
     <t>B4</t>
+  </si>
+  <si>
+    <t>HOODIE.CODE.000113</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>skill_impact_index categories</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>C2</t>
+  </si>
+  <si>
+    <t>C3</t>
+  </si>
+  <si>
+    <t>C4</t>
+  </si>
+  <si>
+    <t>C5</t>
+  </si>
+  <si>
+    <t>C6</t>
+  </si>
+  <si>
+    <t>C7</t>
+  </si>
+  <si>
+    <t>C8</t>
+  </si>
+  <si>
+    <t>C9</t>
+  </si>
+  <si>
+    <t>C10</t>
+  </si>
+  <si>
+    <t>C0</t>
   </si>
 </sst>
 </file>
@@ -449,7 +521,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="37.33203125" style="1" customWidth="1"/>
@@ -612,6 +684,193 @@
         <v>0</v>
       </c>
     </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" t="s">
+        <v>37</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" t="s">
+        <v>37</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" t="s">
+        <v>37</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" t="s">
+        <v>37</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D16" t="s">
+        <v>37</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D17" t="s">
+        <v>37</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D18" t="s">
+        <v>37</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D19" t="s">
+        <v>37</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D20" t="s">
+        <v>37</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>